<commit_message>
feat(project-service): Phase 1 RA — Import Set, catalog artifact và workbook Analysis
Hoàn thiện parse/import Analysis, lifecycle draft→approve, trace gaps và template Requirement_Analysis.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/services/project-service/assets/Requirement_Analysis.xlsx
+++ b/services/project-service/assets/Requirement_Analysis.xlsx
@@ -13,13 +13,18 @@
     <sheet sheetId="7" name="05_FR" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="06_UC" state="visible" r:id="rId11"/>
     <sheet sheetId="9" name="07_NFR" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="08_Scope" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="09_Interfaces" state="visible" r:id="rId14"/>
+    <sheet sheetId="12" name="10_Data" state="visible" r:id="rId15"/>
+    <sheet sheetId="13" name="11_Glossary" state="visible" r:id="rId16"/>
+    <sheet sheetId="14" name="12_Assumptions" state="visible" r:id="rId17"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="220">
   <si>
     <t>Key</t>
   </si>
@@ -36,7 +41,7 @@
     <t>TemplateVersion</t>
   </si>
   <si>
-    <t>2.1-analysis</t>
+    <t>2.2-analysis</t>
   </si>
   <si>
     <t>Language</t>
@@ -60,7 +65,7 @@
     <t>Sheets</t>
   </si>
   <si>
-    <t>01_Traceability (required) + 02_BG … 07_NFR. Trace every Analysis ID back to Customer Requirement ID (CR-* from Raw 03_Requirement).</t>
+    <t>01_Traceability (required) + 02_BG … 07_NFR + optional 08_Scope + 09_Interfaces … 12_Assumptions. Trace Analysis IDs back to Customer Requirement ID (CR-* from Raw 03_Requirement).</t>
   </si>
   <si>
     <t>Flow</t>
@@ -75,6 +80,18 @@
     <t>Leave Target blank unless grounded in customer, standard, or confirmed decision. Do not invent targets.</t>
   </si>
   <si>
+    <t>Scope</t>
+  </si>
+  <si>
+    <t>Optional sheet 08_Scope (Scope Type = In Scope | Out of Scope). Seeded as SCOPE artifacts. Also fill Raw 01_Project_Context In Scope / Out of Scope for customer language.</t>
+  </si>
+  <si>
+    <t>IEEE sheets</t>
+  </si>
+  <si>
+    <t>Optional 09_Interfaces / 10_Data / 11_Glossary / 12_Assumptions seed INTERFACE, DATA, GLOSSARY, ASSUMPTION artifacts (not required for Start Planning gate).</t>
+  </si>
+  <si>
     <t>Analysis ID</t>
   </si>
   <si>
@@ -489,9 +506,6 @@
     <t>Measurement</t>
   </si>
   <si>
-    <t>Scope</t>
-  </si>
-  <si>
     <t>Source</t>
   </si>
   <si>
@@ -514,6 +528,162 @@
   </si>
   <si>
     <t>Target left blank — not confirmed by customer</t>
+  </si>
+  <si>
+    <t>Scope Type</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Date Raised</t>
+  </si>
+  <si>
+    <t>In Scope</t>
+  </si>
+  <si>
+    <t>Students can search and register courses online via web</t>
+  </si>
+  <si>
+    <t>2026-09-01</t>
+  </si>
+  <si>
+    <t>From Raw In Scope</t>
+  </si>
+  <si>
+    <t>Reject registration when class capacity is full</t>
+  </si>
+  <si>
+    <t>University SSO authentication for students/lecturers/admin</t>
+  </si>
+  <si>
+    <t>Integration constraint</t>
+  </si>
+  <si>
+    <t>Out of Scope</t>
+  </si>
+  <si>
+    <t>Native mobile apps (iOS/Android stores)</t>
+  </si>
+  <si>
+    <t>Web responsive only for this release</t>
+  </si>
+  <si>
+    <t>Payment / tuition gateway</t>
+  </si>
+  <si>
+    <t>Interface ID</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Direction</t>
+  </si>
+  <si>
+    <t>Protocol</t>
+  </si>
+  <si>
+    <t>Related Artifact IDs</t>
+  </si>
+  <si>
+    <t>IF-001</t>
+  </si>
+  <si>
+    <t>Campus SSO</t>
+  </si>
+  <si>
+    <t>auth</t>
+  </si>
+  <si>
+    <t>in</t>
+  </si>
+  <si>
+    <t>SAML/OIDC</t>
+  </si>
+  <si>
+    <t>University identity provider for student/lecturer login</t>
+  </si>
+  <si>
+    <t>FR-001;NFR-001</t>
+  </si>
+  <si>
+    <t>Data ID</t>
+  </si>
+  <si>
+    <t>Entity</t>
+  </si>
+  <si>
+    <t>Attributes</t>
+  </si>
+  <si>
+    <t>Rules</t>
+  </si>
+  <si>
+    <t>DATA-001</t>
+  </si>
+  <si>
+    <t>Enrollment</t>
+  </si>
+  <si>
+    <t>studentId; courseId; status; enrolledAt</t>
+  </si>
+  <si>
+    <t>status in {pending,active,rejected}; unique(studentId,courseId)</t>
+  </si>
+  <si>
+    <t>FR-001;UC-001</t>
+  </si>
+  <si>
+    <t>Term ID</t>
+  </si>
+  <si>
+    <t>Term</t>
+  </si>
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <t>GL-001</t>
+  </si>
+  <si>
+    <t>SSO</t>
+  </si>
+  <si>
+    <t>Single Sign-On via campus identity provider</t>
+  </si>
+  <si>
+    <t>GL-002</t>
+  </si>
+  <si>
+    <t>Capacity</t>
+  </si>
+  <si>
+    <t>Maximum seats allowed for a course section</t>
+  </si>
+  <si>
+    <t>Assumption ID</t>
+  </si>
+  <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>Impact If Invalid</t>
+  </si>
+  <si>
+    <t>ASM-001</t>
+  </si>
+  <si>
+    <t>Campus SSO is available for all enrolled students at go-live</t>
+  </si>
+  <si>
+    <t>Registration must fall back to local accounts; timeline slips</t>
+  </si>
+  <si>
+    <t>IF-001;BG-001</t>
   </si>
 </sst>
 </file>
@@ -931,9 +1101,424 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" t="s">
+        <v>173</v>
+      </c>
+      <c r="F3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" t="s">
+        <v>173</v>
+      </c>
+      <c r="F4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>178</v>
+      </c>
+      <c r="B5" t="s">
+        <v>179</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" t="s">
+        <v>173</v>
+      </c>
+      <c r="F5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>178</v>
+      </c>
+      <c r="B6" t="s">
+        <v>181</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
+        <v>173</v>
+      </c>
+      <c r="F6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D1" t="s">
+        <v>185</v>
+      </c>
+      <c r="E1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G1" t="s">
+        <v>187</v>
+      </c>
+      <c r="H1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" t="s">
+        <v>61</v>
+      </c>
+      <c r="J1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E2" t="s">
+        <v>192</v>
+      </c>
+      <c r="F2" t="s">
+        <v>193</v>
+      </c>
+      <c r="G2" t="s">
+        <v>194</v>
+      </c>
+      <c r="H2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E2" t="s">
+        <v>203</v>
+      </c>
+      <c r="F2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1" t="s">
+        <v>206</v>
+      </c>
+      <c r="D1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" t="s">
+        <v>215</v>
+      </c>
+      <c r="D1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C2" t="s">
+        <v>218</v>
+      </c>
+      <c r="D2" t="s">
+        <v>219</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -974,6 +1559,22 @@
       </c>
       <c r="B5" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -989,186 +1590,186 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" t="s">
         <v>32</v>
       </c>
-      <c r="B3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" t="s">
-        <v>28</v>
-      </c>
       <c r="E3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" t="s">
         <v>34</v>
       </c>
-      <c r="F3" t="s">
-        <v>30</v>
-      </c>
       <c r="G3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" t="s">
         <v>34</v>
       </c>
-      <c r="F4" t="s">
-        <v>30</v>
-      </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" t="s">
         <v>34</v>
       </c>
-      <c r="F6" t="s">
-        <v>30</v>
-      </c>
       <c r="G6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
         <v>41</v>
       </c>
-      <c r="B7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" t="s">
-        <v>37</v>
-      </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" t="s">
         <v>34</v>
       </c>
-      <c r="F7" t="s">
-        <v>30</v>
-      </c>
       <c r="G7" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1184,78 +1785,78 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="J1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="K1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="L1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="I2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="K2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="L2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1271,84 +1872,84 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="I1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="J1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="K1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="L1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="M1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E2" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="I2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="J2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="K2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="L2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="M2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1364,152 +1965,152 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="J1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="K1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="L1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="M1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="N1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="O1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="P1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="I2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="J2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="K2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="L2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="M2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="O2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="P2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F3" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="G3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H3" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I3" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="J3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="K3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="L3" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="M3" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="N3" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="O3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="P3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1525,464 +2126,464 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="D1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="E1" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="F1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="H1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="J1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="K1" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="L1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="M1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="N1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="O1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="P1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="Q1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="R1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="S1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="T1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="U1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="V1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="W1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="X1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="Y1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" t="s">
         <v>31</v>
       </c>
-      <c r="C2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D2" t="s">
-        <v>117</v>
-      </c>
-      <c r="E2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H2" t="s">
-        <v>27</v>
-      </c>
       <c r="I2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="J2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="K2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="L2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="M2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="O2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="P2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="Q2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="S2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="T2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="U2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="V2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="W2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="X2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="Y2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B3" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D3" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="E3" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="I3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="K3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="L3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="M3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="O3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="P3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="Q3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="S3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="T3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="U3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="V3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="W3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="X3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="Y3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="E4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J4" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="K4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="L4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="M4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="O4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="P4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="Q4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="R4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="S4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="T4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="U4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="V4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="W4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="X4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="Y4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D5" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="E5" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F5" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G5" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J5" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="K5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="L5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="M5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N5" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="O5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="P5" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="Q5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="R5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="S5" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="T5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="U5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="V5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="W5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="X5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="Y5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C6" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="E6" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F6" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H6" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="I6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J6" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="K6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="L6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="M6" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="N6" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="O6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="P6" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="Q6" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="R6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="S6" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="T6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="U6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="V6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="W6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="X6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="Y6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1998,126 +2599,126 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B1" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E1" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G1" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="H1" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="I1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="J1" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="K1" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L1" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="M1" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="N1" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="O1" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="P1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="Q1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="R1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="S1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="T1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" t="s">
         <v>41</v>
       </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D2" t="s">
-        <v>37</v>
-      </c>
       <c r="E2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="G2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="H2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="I2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="J2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="K2" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="L2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="M2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="N2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="O2" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="P2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="Q2" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="R2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="S2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="T2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -2133,84 +2734,84 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C1" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E1" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F1" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H1" t="s">
-        <v>156</v>
+        <v>18</v>
       </c>
       <c r="I1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="J1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="K1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="L1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="M1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="H2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="I2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="J2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="L2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="M2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>